<commit_message>
Add P16 computer pun and its twin N16 to the test set
</commit_message>
<xml_diff>
--- a/evaluation/Group8_Pun_Test_Set.xlsx
+++ b/evaluation/Group8_Pun_Test_Set.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1780,9 +1780,99 @@
       </c>
       <c r="L31" s="3" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>I don't enjoy computer puns one bit.</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Pun</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Homographic pun</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>binary digit</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>the smallest amount (not at all)</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="5" t="n"/>
+      <c r="J32" s="5" t="n"/>
+      <c r="K32" s="3">
+        <f>IF(J32="","",IF(AND(C32="Pun",J32="Pun"),"TP",IF(AND(C32="Non-pun",J32="Pun"),"FP",IF(AND(C32="Pun",J32="Non-pun"),"FN","TN"))))</f>
+        <v/>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Added Oct 16. Stages 1-2 call it a pun for the wrong reason: they pick 'computer', not 'bit', and also flag its twin N16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>N16</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>I don't enjoy computer puns at all.</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Non-pun</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>De-punned twin</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
+      <c r="K33" s="3">
+        <f>IF(J33="","",IF(AND(C33="Pun",J33="Pun"),"TP",IF(AND(C33="Non-pun",J33="Pun"),"FP",IF(AND(C33="Pun",J33="Non-pun"),"FN","TN"))))</f>
+        <v/>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Second reading removed ('one bit' becomes 'at all').</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:J31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:J33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pun,Non-pun"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1812,6 +1902,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1819,7 +1910,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF('Test Set'!K2:K31,"TP")</f>
+        <f>COUNTIF('Test Set'!K2:K33,"TP")</f>
         <v/>
       </c>
     </row>
@@ -1830,7 +1921,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF('Test Set'!K2:K31,"FP")</f>
+        <f>COUNTIF('Test Set'!K2:K33,"FP")</f>
         <v/>
       </c>
     </row>
@@ -1841,7 +1932,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF('Test Set'!K2:K31,"FN")</f>
+        <f>COUNTIF('Test Set'!K2:K33,"FN")</f>
         <v/>
       </c>
     </row>
@@ -1852,7 +1943,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF('Test Set'!K2:K31,"TN")</f>
+        <f>COUNTIF('Test Set'!K2:K33,"TN")</f>
         <v/>
       </c>
     </row>
@@ -1915,7 +2006,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>IFERROR(COUNTIFS('Test Set'!D2:D31,"Homographic pun",'Test Set'!K2:K31,"TP")/COUNTIFS('Test Set'!D2:D31,"Homographic pun",'Test Set'!J2:J31,"&lt;&gt;"),"n/a")</f>
+        <f>IFERROR(COUNTIFS('Test Set'!D2:D33,"Homographic pun",'Test Set'!K2:K33,"TP")/COUNTIFS('Test Set'!D2:D33,"Homographic pun",'Test Set'!J2:J33,"&lt;&gt;"),"n/a")</f>
         <v/>
       </c>
     </row>
@@ -1926,7 +2017,7 @@
         </is>
       </c>
       <c r="B14" s="8">
-        <f>IFERROR(COUNTIFS('Test Set'!D2:D31,"Heterographic*",'Test Set'!K2:K31,"TP")/COUNTIFS('Test Set'!D2:D31,"Heterographic*",'Test Set'!J2:J31,"&lt;&gt;"),"n/a")</f>
+        <f>IFERROR(COUNTIFS('Test Set'!D2:D33,"Heterographic*",'Test Set'!K2:K33,"TP")/COUNTIFS('Test Set'!D2:D33,"Heterographic*",'Test Set'!J2:J33,"&lt;&gt;"),"n/a")</f>
         <v/>
       </c>
     </row>
@@ -1941,10 +2032,11 @@
         </is>
       </c>
       <c r="B16" s="8">
-        <f>IFERROR(SUMPRODUCT(('Test Set'!I2:I31&lt;&gt;"")*('Test Set'!I2:I31='Test Set'!C2:C31))/COUNTA('Test Set'!I2:I31),"n/a")</f>
-        <v/>
-      </c>
-    </row>
+        <f>IFERROR(SUMPRODUCT(('Test Set'!I2:I33&lt;&gt;"")*('Test Set'!I2:I33='Test Set'!C2:C33))/COUNTA('Test Set'!I2:I33),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
@@ -1969,7 +2061,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>3. Counts are small (15 + 15), so one error moves a rate by about 7 points. Report the raw counts alongside the percentages.</t>
+          <t>3. Counts are small (16 + 16), so one error moves a rate by about 6 points. Report the raw counts alongside the percentages.</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2627,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
@@ -2587,7 +2678,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>

</xml_diff>